<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.001-06 Les moufles de Nina
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.001-06.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.001-06.xlsx
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nina, papa, maman, maîtresse</t>
+          <t>Nina, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nina veut réchauffer ses moufles, puis poser son crayon rouge. L'air pique. Un chuchotement serre son ventre. Le soir, elle raconte, et le nuage des moufles revient sur le radiateur.</t>
+          <t>Sur le pouce, un éclat de moufle brille. Nina veut les moufles, maintenant. Elle tire trop vite : une moufle tombe. À l'école, un camarade veut le secret tout de suite. Elle coupe la classe : les mots se perdent. Le soir, elle ouvre la bouche trop vite. Elle refuse de foncer, attend, raconte. Merci vécu. L'éclat de moufle tient sur le pouce.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Les moufles sèchent sur le radiateur. Elles font un tout petit nuage, tout blanc. La laine sent le froid d'en dehors. La fenêtre tremble un peu. Papa pose le cartable contre le mur. Maman boutonne le manteau, une, deux, trois. Ça sent la soupe qui attend dans la casserole. Les moufles fument, tu vois ? La laine redevient douce. En ce moment, Nina pose sa joue près de la laine tiède. C'est chaud, maman. Encore un moment, puis on part. Je veux dessiner le nuage des moufles. Avec le crayon rouge. Le crayon est dans la pochette. Tes deux mains seront au chaud. Le bouton du haut est bien fermé ? Oui, maman. Un, deux, trois. Nina enfile les moufles. La laine est douce, encore tiède. Dehors, l'air pique un peu le nez. Les pas sonnent sur les cailloux gelés. On tient la main. L'école est plus chaude que la rue. Ça sent les manteaux mouillés, près des crochets. Bonjour. On range les crayons. Bonjour, maîtresse. Nina écoute. Elle range son crayon rouge, tout droit. Le rouge tape un petit coup dans la boîte. Merci, Nina. Vous avez bien écouté. Plus tard, quelqu'un s'approche. Une voix parle tout bas, d'un secret. Nina sent un malaise. Son ventre se serre. Elle garde les mains sur la table. Elle reste près de sa chaise. Le soir, les moufles sont sèches, toutes douces. La porte s'ouvre. Te voilà. Le manteau est lourd de froid. Nina pose les moufles sur le radiateur. Le petit nuage revient. Le ventre est encore serré.</t>
+          <t>La fenêtre tremble contre le bois. Dehors, le froid pique les vitres. Dans l'entrée, un petit nuage blanc s'élève. Les moufles sèchent sur le radiateur. La laine sent le froid de la rue. Sur le pouce, un éclat de moufle brille. Il est petit, maman. C'est le chaud qui revient. Le cartable est contre le mur. Papa pose le cartable, bien droit. Maman boutonne le manteau, une, deux, trois. Ça sent la soupe, dans la casserole. Les moufles, maintenant ! Elles fument un peu, Nina. Je les prends ! En ce moment, Nina saisit les deux moufles. La laine reste humide, un peu lourde. Elle tire trop vite. Une moufle glisse, tombe. L'éclat de moufle tremble, puis tient. Oh. Le sourire de Nina disparaît. Dans sa poitrine, envie et inquiétude se bousculent. Ça ne veut pas. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu veux les mains au chaud ? Oui, papa. On les met dehors, d'accord ? D'accord. Nina enfile les moufles, plus lente. La laine colle un peu aux doigts. Le bouton du haut ? Fermé. Dehors, l'air pique le nez. Les pas sonnent sur les cailloux gelés. Papa tient sa main. L'école est plus chaude que la rue. Ça sent les manteaux mouillés, près des crochets. Nina pose le cartable contre le casier. La classe pose une histoire, près du tableau. Nina écoute, les mains sur la table. Un camarade s'approche. Regarde, maintenant. C'est un secret. Il parle trop près de son oreille. Nina veut écouter la classe. Le camarade veut le secret, maintenant. Nina sent un malaise. Son ventre se serre. Je le dis, maintenant ! Elle ouvre la bouche trop vite. Ses mots se cognent à ceux de la classe. Personne ne tourne la tête. Oh. Nina referme la bouche. Elle garde les mains sur la table. Le soir, la porte s'ouvre. Le manteau est lourd de froid. Te voilà, Nina. Les moufles sont sèches, sur le radiateur. Le petit nuage n'est plus là. Nina pose les moufles près du métal. Elle ouvre la bouche.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Les moufles sèchent sur le radiateur. Elles font un tout petit nuage, tout blanc. La laine sent le froid d'en dehors. La fenêtre tremble un peu. Papa pose le cartable contre le mur. Maman boutonne le manteau, une, deux, trois. Ça sent la soupe qui attend dans la casserole. Les moufles fument, tu vois ? La laine redevient douce. En ce moment, Nina pose sa joue près de la laine tiède. C'est chaud, maman. Encore un moment, puis on part. Je veux dessiner le nuage des moufles. Avec le crayon rouge. Le crayon est dans la pochette. Tes deux mains seront au chaud. Le bouton du haut est bien fermé ? Oui, maman. Un, deux, trois. Nina enfile les moufles. La laine est douce, encore tiède. Dehors, l'air pique un peu le nez. Les pas sonnent sur les cailloux gelés. On tient la main. L'école est plus chaude que la rue. Ça sent les manteaux mouillés, près des crochets. Bonjour. On range les crayons. Bonjour, maîtresse. Nina écoute. Elle range son crayon rouge, tout droit. Le rouge tape un petit coup dans la boîte. Merci, Nina. Vous avez bien écouté. Plus tard, quelqu'un s'approche. Une voix parle tout bas, d'un secret. Nina sent un malaise. Son ventre se serre. Elle garde les mains sur la table. Elle reste près de sa chaise. Le soir, les moufles sont sèches, toutes douces. La porte s'ouvre. Te voilà. Le manteau est lourd de froid. Nina pose les moufles sur le radiateur. Le petit nuage revient. Le ventre est encore serré.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La fenêtre tremble contre le bois. Dehors, le froid pique les vitres. Dans l'entrée, un petit nuage blanc s'élève. Les moufles sèchent sur le radiateur. La laine sent le froid de la rue. Sur le pouce, un &lt;emphasis level="moderate"&gt;éclat de moufle&lt;/emphasis&gt; brille. Il est petit, maman. C'est le chaud qui revient. Le cartable est contre le mur. Papa pose le cartable, bien droit. Maman boutonne le manteau, une, deux, trois. Ça sent la soupe, dans la casserole. Les moufles, maintenant ! Elles fument un peu, Nina. Je les prends ! En ce moment, Nina saisit les deux moufles. La laine reste humide, un peu lourde. Elle tire trop vite. Une moufle glisse, tombe. L'éclat de moufle tremble, puis tient. Oh. Le sourire de Nina disparaît. Dans sa poitrine, envie et inquiétude se bousculent. Ça ne veut pas. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu veux les mains au chaud ? Oui, papa. On les met dehors, d'accord ? D'accord. Nina enfile les moufles, plus lente. La laine colle un peu aux doigts. Le bouton du haut ? Fermé. Dehors, l'air pique le nez. Les pas sonnent sur les cailloux gelés. Papa tient sa main. L'école est plus chaude que la rue. Ça sent les manteaux mouillés, près des crochets. Nina pose le cartable contre le casier. La classe pose une histoire, près du tableau. Nina écoute, les mains sur la table. Un camarade s'approche. Regarde, maintenant. C'est un secret. Il parle trop près de son oreille. Nina veut écouter la classe. Le camarade veut le secret, maintenant. Nina sent un malaise. Son ventre se serre. Je le dis, maintenant ! Elle ouvre la bouche trop vite. Ses mots se cognent à ceux de la classe. Personne ne tourne la tête. Oh. Nina referme la bouche. Elle garde les mains sur la table. Le soir, la porte s'ouvre. Le manteau est lourd de froid. Te voilà, Nina. Les moufles sont sèches, sur le radiateur. Le petit nuage n'est plus là. Nina pose les moufles près du métal. Elle ouvre la bouche.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Xavier est à l'école. La maîtresse parle. Xavier aime &lt;emphasis&gt;écouter&lt;/emphasis&gt;. La maîtresse dit : on range les crayons. Xavier range son crayon. Il écoute bien. Plus tard, un camarade chuchote. Il dit : c'est un secret. Garde ça pour toi. Xavier sent un malaise. Son ventre est serré. Le soir, maman l'attend. Xavier vient raconter à la maison. Il dit : maman, j'ai eu un malaise. Un camarade a parlé d'un secret. Maman l'écoute. Maman dit : tu as bien fait. On aime écouter la maîtresse. Si tu as un malaise, tu viens raconter à papa ou maman. [pause]</t>
+          <t>La fenêtre tremble contre le bois. Dehors, le froid pique les vitres. Dans l'entrée, un petit nuage blanc s'élève. Les moufles sèchent sur le radiateur. La laine sent le froid de la rue. Sur le pouce, un &lt;emphasis&gt;éclat de moufle&lt;/emphasis&gt; brille. Il est petit, maman. C'est le chaud qui revient. Le cartable est contre le mur. Papa pose le cartable, bien droit. Maman boutonne le manteau, une, deux, trois. Ça sent la soupe, dans la casserole. Les moufles, maintenant ! Elles fument un peu, Nina. Je les prends ! En ce moment, Nina saisit les deux moufles. La laine reste humide, un peu lourde. Elle tire trop vite. Une moufle glisse, tombe. L'éclat de moufle tremble, puis tient. Oh. Le sourire de Nina disparaît. Dans sa poitrine, envie et inquiétude se bousculent. Ça ne veut pas. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu veux les mains au chaud ? Oui, papa. On les met dehors, d'accord ? D'accord. Nina enfile les moufles, plus lente. La laine colle un peu aux doigts. Le bouton du haut ? Fermé. Dehors, l'air pique le nez. Les pas sonnent sur les cailloux gelés. Papa tient sa main. L'école est plus chaude que la rue. Ça sent les manteaux mouillés, près des crochets. Nina pose le cartable contre le casier. La classe pose une histoire, près du tableau. Nina écoute, les mains sur la table. Un camarade s'approche. Regarde, maintenant. C'est un secret. Il parle trop près de son oreille. Nina veut écouter la classe. Le camarade veut le secret, maintenant. Nina sent un malaise. Son ventre se serre. Je le dis, maintenant ! Elle ouvre la bouche trop vite. Ses mots se cognent à ceux de la classe. Personne ne tourne la tête. Oh. Nina referme la bouche. Elle garde les mains sur la table. Le soir, la porte s'ouvre. Le manteau est lourd de froid. Te voilà, Nina. Les moufles sont sèches, sur le radiateur. Le petit nuage n'est plus là. Nina pose les moufles près du métal. Elle ouvre la bouche. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>écouter</t>
+          <t>éclat de moufle</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,61 +1321,82 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_les_moufles_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Les moufles sèchent sur le radiateur.
-narrateur|Elles font un tout petit nuage, tout blanc.
-narrateur|La laine sent le froid d'en dehors.
-narrateur|La fenêtre tremble un peu.
-narrateur|Papa pose le cartable contre le mur.
+          <t>narrateur|La fenêtre tremble contre le bois.
+narrateur|Dehors, le froid pique les vitres.
+narrateur|Dans l'entrée, un petit nuage blanc s'élève.
+narrateur|Les moufles sèchent sur le radiateur.
+narrateur|La laine sent le froid de la rue.
+narrateur|Sur le pouce, un éclat de moufle brille.
+enfant-f|Il est petit, maman.
+maman|C'est le chaud qui revient.
+papa|Le cartable est contre le mur.
+narrateur|Papa pose le cartable, bien droit.
 narrateur|Maman boutonne le manteau, une, deux, trois.
-narrateur|Ça sent la soupe qui attend dans la casserole.
-papa|Les moufles fument, tu vois ?
-maman|La laine redevient douce.
-narrateur|En ce moment, Nina pose sa joue près de la laine tiède.
-enfant-f|C'est chaud, maman.
-maman|Encore un moment, puis on part.
-enfant-f|Je veux dessiner le nuage des moufles.
-enfant-f|Avec le crayon rouge.
-papa|Le crayon est dans la pochette.
-papa|Tes deux mains seront au chaud.
-maman|Le bouton du haut est bien fermé ?
-enfant-f|Oui, maman.
-enfant-f|Un, deux, trois.
-narrateur|Nina enfile les moufles.
-narrateur|La laine est douce, encore tiède.
-narrateur|Dehors, l'air pique un peu le nez.
+narrateur|Ça sent la soupe, dans la casserole.
+enfant-f|Les moufles, maintenant !
+maman|Elles fument un peu, Nina.
+enfant-f|Je les prends !
+narrateur|En ce moment, Nina saisit les deux moufles.
+narrateur|La laine reste humide, un peu lourde.
+narrateur|Elle tire trop vite.
+narrateur|Une moufle glisse, tombe.
+narrateur|L'éclat de moufle tremble, puis tient.
+enfant-f|Oh.
+narrateur|Le sourire de Nina disparaît.
+narrateur|Dans sa poitrine, envie et inquiétude se bousculent.
+enfant-f|Ça ne veut pas.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa se baisse à sa hauteur.
+papa|Tu veux les mains au chaud ?
+enfant-f|Oui, papa.
+maman|On les met dehors, d'accord ?
+enfant-f|D'accord.
+narrateur|Nina enfile les moufles, plus lente.
+narrateur|La laine colle un peu aux doigts.
+papa|Le bouton du haut ?
+enfant-f|Fermé.
+narrateur|Dehors, l'air pique le nez.
 narrateur|Les pas sonnent sur les cailloux gelés.
-maman|On tient la main.
+narrateur|Papa tient sa main.
 narrateur|L'école est plus chaude que la rue.
 narrateur|Ça sent les manteaux mouillés, près des crochets.
-maitresse|Bonjour.
-maitresse|On range les crayons.
-enfant-f|Bonjour, maîtresse.
-narrateur|Nina écoute.
-narrateur|Elle range son crayon rouge, tout droit.
-narrateur|Le rouge tape un petit coup dans la boîte.
-maitresse|Merci, Nina.
-maitresse|Vous avez bien écouté.
-narrateur|Plus tard, quelqu'un s'approche.
-narrateur|Une voix parle tout bas, d'un secret.
+narrateur|Nina pose le cartable contre le casier.
+narrateur|La classe pose une histoire, près du tableau.
+narrateur|Nina écoute, les mains sur la table.
+narrateur|Un camarade s'approche.
+copain|Regarde, maintenant.
+copain|C'est un secret.
+narrateur|Il parle trop près de son oreille.
+narrateur|Nina veut écouter la classe.
+narrateur|Le camarade veut le secret, maintenant.
 narrateur|Nina sent un malaise.
 narrateur|Son ventre se serre.
+enfant-f|Je le dis, maintenant !
+narrateur|Elle ouvre la bouche trop vite.
+narrateur|Ses mots se cognent à ceux de la classe.
+narrateur|Personne ne tourne la tête.
+enfant-f|Oh.
+narrateur|Nina referme la bouche.
 narrateur|Elle garde les mains sur la table.
-narrateur|Elle reste près de sa chaise.
-narrateur|Le soir, les moufles sont sèches, toutes douces.
-narrateur|La porte s'ouvre.
-maman|Te voilà.
-maman|Le manteau est lourd de froid.
-narrateur|Nina pose les moufles sur le radiateur.
-narrateur|Le petit nuage revient.
-narrateur|Le ventre est encore serré.</t>
+narrateur|Le soir, la porte s'ouvre.
+narrateur|Le manteau est lourd de froid.
+maman|Te voilà, Nina.
+papa|Les moufles sont sèches, sur le radiateur.
+narrateur|Le petit nuage n'est plus là.
+narrateur|Nina pose les moufles près du métal.
+narrateur|Elle ouvre la bouche.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>pluie,porte</t>
+          <t>radiateur,laine</t>
         </is>
       </c>
     </row>
@@ -1407,12 +1428,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nina a un malaise. Que fait-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nina a un &lt;emphasis level="moderate"&gt;malaise&lt;/emphasis&gt;. Que fait-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Xavier a un malaise. Que fait-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nina a un &lt;emphasis&gt;malaise&lt;/emphasis&gt;. Que fait-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1475,7 +1496,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1486,7 +1507,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1501,34 +1522,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>malaise</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1543,17 +1568,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_attend_puis_raconte; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1586,17 +1611,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Maman. J'ai eu un malaise. Quelqu'un a parlé d'un secret. On t'écoute. Viens près de la soupe. Nina parle. Maman écoute. Papa écoute. Tu as bien fait de raconter. À l'école, on écoute la maîtresse. Si tu as un malaise, tu viens le dire. Le ventre de Nina se desserre, tout doucement.</t>
+          <t>Nina ouvre la bouche trop vite. Maman, un secret. Maman n'a pas fini sa phrase. Le manteau est lourd, Nina. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Nina refuse de foncer. Elle referme la bouche. Elle pose les mains à plat. Elle écoute l'entrée, un instant. Les moufles sèchent près du radiateur. Papa pose le cartable contre le mur. La soupe fume un peu. Maman n'a pas fini non plus. Nina attend que le silence arrive. Sur le pouce, l'éclat de moufle brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Un camarade a parlé d'un secret. Mon ventre s'est serré. Merci, Nina. Papa a entendu toute la phrase. Tu veux ta soupe ? Oui, maman. Le ventre de Nina se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Maman. J'ai eu un malaise. Quelqu'un a parlé d'un secret. On t'écoute. Viens près de la soupe. Nina parle. Maman écoute. Papa écoute. Tu as bien fait de raconter. À l'école, on écoute la maîtresse. Si tu as un malaise, tu viens le dire. Le ventre de Nina se desserre, tout doucement.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina ouvre la bouche trop vite. Maman, un &lt;emphasis level="moderate"&gt;secret&lt;/emphasis&gt;. Maman n'a pas fini sa phrase. Le manteau est lourd, Nina. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Nina refuse de foncer. Elle referme la bouche. Elle pose les mains à plat. Elle écoute l'entrée, un instant. Les moufles sèchent près du radiateur. Papa pose le cartable contre le mur. La soupe fume un peu. Maman n'a pas fini non plus. Nina attend que le silence arrive. Sur le pouce, l'éclat de moufle brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Un camarade a parlé d'un secret. Mon ventre s'est serré. Merci, Nina. Papa a entendu toute la phrase. Tu veux ta soupe ? Oui, maman. Le ventre de Nina se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Xavier a écouté la maîtresse. Il a raconté son malaise à la maison. Maman est là. [pause]</t>
+          <t>Nina ouvre la bouche trop vite. Maman, un &lt;emphasis&gt;secret&lt;/emphasis&gt;. Maman n'a pas fini sa phrase. Le manteau est lourd, Nina. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Nina refuse de foncer. Elle referme la bouche. Elle pose les mains à plat. Elle écoute l'entrée, un instant. Les moufles sèchent près du radiateur. Papa pose le cartable contre le mur. La soupe fume un peu. Maman n'a pas fini non plus. Nina attend que le silence arrive. Sur le pouce, l'éclat de moufle brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Un camarade a parlé d'un secret. Mon ventre s'est serré. Merci, Nina. Papa a entendu toute la phrase. Tu veux ta soupe ? Oui, maman. Le ventre de Nina se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1643,7 +1668,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1651,10 +1676,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1675,28 +1700,32 @@
       <c r="AG4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>secret</t>
+        </is>
+      </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1705,10 +1734,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1721,23 +1750,43 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_attend_puis_on_l_entend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-f|Maman.
-enfant-f|J'ai eu un malaise.
-enfant-f|Quelqu'un a parlé d'un secret.
-maman|On t'écoute.
-papa|Viens près de la soupe.
-narrateur|Nina parle.
-narrateur|Maman écoute.
-narrateur|Papa écoute.
-maman|Tu as bien fait de raconter.
-papa|À l'école, on écoute la maîtresse.
-maman|Si tu as un malaise, tu viens le dire.
-narrateur|Le ventre de Nina se desserre, tout doucement.</t>
+          <t>narrateur|Nina ouvre la bouche trop vite.
+enfant-f|Maman, un secret.
+narrateur|Maman n'a pas fini sa phrase.
+maman|Le manteau est lourd, Nina.
+narrateur|Les deux voix se mélangent.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Nina refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Elle pose les mains à plat.
+narrateur|Elle écoute l'entrée, un instant.
+papa|Les moufles sèchent près du radiateur.
+narrateur|Papa pose le cartable contre le mur.
+maman|La soupe fume un peu.
+narrateur|Maman n'a pas fini non plus.
+narrateur|Nina attend que le silence arrive.
+narrateur|Sur le pouce, l'éclat de moufle brille.
+enfant-f|Il est là.
+enfant-f|Je peux te dire quelque chose ?
+maman|Oui, nous t'écoutons.
+enfant-f|Un camarade a parlé d'un secret.
+enfant-f|Mon ventre s'est serré.
+papa|Merci, Nina.
+narrateur|Papa a entendu toute la phrase.
+maman|Tu veux ta soupe ?
+enfant-f|Oui, maman.
+narrateur|Le ventre de Nina se desserre.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>soupe,moufles</t>
         </is>
       </c>
     </row>
@@ -1764,17 +1813,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Maman verse la soupe. La vapeur fait de la buée. Tu as tes deux mains libres ? Oui, papa. Nina souffle sur la cuillère. C'est chaud, comme les moufles. Tu as fini ta bolée ? Presque. Nina pose encore la joue près de la laine. Le nuage est revenu. On le laisse sécher. La fenêtre tremble moins. La cuisine est calme. Merci, maman. Merci, papa.</t>
+          <t>Nina veut tout dire, d'un coup. Elle prend la cuillère et les moufles. La cuillère tape le bol. Une moufle glisse vers le sol. Ça tombe ! Nina veut foncer, d'un coup. Nina refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Elle regarde les moufles. Elle écoute le radiateur, un instant. Le métal fait un petit bruit. Sur le pouce, l'éclat de moufle brille. Comme ce matin ! Tu le vois, toi ? Oui, sur cette laine. Nina pose la cuillère, d'abord. Puis elle glisse les moufles au chaud. La soupe, Nina ? Oui. Elle s'assoit. Le bol est lisse, un peu lourd. Elle boit une gorgée. La soupe est tiède.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Maman verse la soupe. La vapeur fait de la buée. Tu as tes deux mains libres ? Oui, papa. Nina souffle sur la cuillère. C'est chaud, comme les moufles. Tu as fini ta bolée ? Presque. Nina pose encore la joue près de la laine. Le nuage est revenu. On le laisse sécher. La fenêtre tremble moins. La cuisine est calme. Merci, maman. Merci, papa.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina veut tout dire, d'un coup. Elle prend la cuillère et les moufles. La cuillère tape le bol. Une moufle glisse vers le sol. Ça tombe ! Nina veut foncer, d'un coup. Nina refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Elle regarde les moufles. Elle écoute le radiateur, un instant. Le métal fait un petit bruit. Sur le pouce, l'&lt;emphasis level="moderate"&gt;éclat de moufle&lt;/emphasis&gt; brille. Comme ce matin ! Tu le vois, toi ? Oui, sur cette laine. Nina pose la cuillère, d'abord. Puis elle glisse les moufles au chaud. La soupe, Nina ? Oui. Elle s'assoit. Le bol est lisse, un peu lourd. Elle boit une gorgée. La soupe est tiède.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Xavier boit un verre d'eau. Maman lui tient la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>&lt;low-pitch&gt;Nina veut tout dire, d'un coup. Elle prend la cuillère et les moufles. La cuillère tape le bol. Une moufle glisse vers le sol. Ça tombe ! Nina veut foncer, d'un coup. Nina refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Elle regarde les moufles. Elle écoute le radiateur, un instant. Le métal fait un petit bruit. Sur le pouce, l'&lt;emphasis&gt;éclat de moufle&lt;/emphasis&gt; brille. Comme ce matin ! Tu le vois, toi ? Oui, sur cette laine. Nina pose la cuillère, d'abord. Puis elle glisse les moufles au chaud. La soupe, Nina ? Oui. Elle s'assoit. Le bol est lisse, un peu lourd. Elle boit une gorgée. La soupe est tiède.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1821,7 +1870,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1829,22 +1878,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1855,30 +1908,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de moufle</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1887,38 +1940,57 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Maman verse la soupe.
-narrateur|La vapeur fait de la buée.
-papa|Tu as tes deux mains libres ?
-enfant-f|Oui, papa.
-narrateur|Nina souffle sur la cuillère.
-narrateur|C'est chaud, comme les moufles.
-maman|Tu as fini ta bolée ?
-enfant-f|Presque.
-narrateur|Nina pose encore la joue près de la laine.
-enfant-f|Le nuage est revenu.
-papa|On le laisse sécher.
-narrateur|La fenêtre tremble moins.
-narrateur|La cuisine est calme.
-enfant-f|Merci, maman.
-enfant-f|Merci, papa.</t>
+          <t>narrateur|Nina veut tout dire, d'un coup.
+narrateur|Elle prend la cuillère et les moufles.
+narrateur|La cuillère tape le bol.
+narrateur|Une moufle glisse vers le sol.
+enfant-f|Ça tombe !
+narrateur|Nina veut foncer, d'un coup.
+narrateur|Nina refuse de foncer.
+narrateur|Ses épaules se serrent un peu.
+narrateur|Ça tape, dans sa poitrine.
+narrateur|Personne ne dit la suite.
+narrateur|Elle regarde les moufles.
+narrateur|Elle écoute le radiateur, un instant.
+narrateur|Le métal fait un petit bruit.
+narrateur|Sur le pouce, l'éclat de moufle brille.
+enfant-f|Comme ce matin !
+papa|Tu le vois, toi ?
+enfant-f|Oui, sur cette laine.
+narrateur|Nina pose la cuillère, d'abord.
+narrateur|Puis elle glisse les moufles au chaud.
+maman|La soupe, Nina ?
+enfant-f|Oui.
+narrateur|Elle s'assoit.
+narrateur|Le bol est lisse, un peu lourd.
+narrateur|Elle boit une gorgée.
+narrateur|La soupe est tiède.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>cuillere,bol</t>
         </is>
       </c>
     </row>
@@ -1945,17 +2017,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Les moufles reposent, toutes douces. La soupe n'envoie plus de nuage. On t'a écoutée, Nina. Tes mains sont au chaud.</t>
+          <t>Les moufles reposent sur le radiateur. Le petit nuage n'est plus là. L'éclat est là, papa. Tu le vois sur le pouce ? Oui, papa. On est bien, ici. La soupe fume un peu, près de la fenêtre. La fenêtre tremble moins. J'ai dit le secret. On t'a entendue, Nina. Oui, maman. Nina pose la joue près de la laine. La laine est tiède, un peu rêche. C'est chaud. Dehors, le froid reste sur les cailloux. L'éclat de moufle tient sur le pouce.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Les moufles reposent, toutes douces. La soupe n'envoie plus de nuage. On t'a écoutée, Nina. Tes mains sont au chaud.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les moufles reposent sur le radiateur. Le petit nuage n'est plus là. L'éclat est là, papa. Tu le vois sur le pouce ? Oui, papa. On est bien, ici. La soupe fume un peu, près de la fenêtre. La fenêtre tremble moins. J'ai dit le secret. On t'a entendue, Nina. Oui, maman. Nina pose la joue près de la laine. La laine est tiède, un peu rêche. C'est chaud. Dehors, le froid reste sur les cailloux. L'&lt;emphasis level="moderate"&gt;éclat de moufle&lt;/emphasis&gt; tient sur le pouce.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les moufles reposent sur le radiateur. Le petit nuage n'est plus là. L'éclat est là, papa. Tu le vois sur le pouce ? Oui, papa. On est bien, ici. La soupe fume un peu, près de la fenêtre. La fenêtre tremble moins. J'ai dit le secret. On t'a entendue, Nina. Oui, maman. Nina pose la joue près de la laine. La laine est tiède, un peu rêche. C'est chaud. Dehors, le froid reste sur les cailloux. L'&lt;emphasis&gt;éclat de moufle&lt;/emphasis&gt; tient sur le pouce.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2002,7 +2074,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2010,10 +2082,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2022,12 +2094,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2036,17 +2108,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de moufle</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2055,11 +2131,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2068,27 +2144,48 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_pouce; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Les moufles reposent, toutes douces.
-narrateur|La soupe n'envoie plus de nuage.
-maman|On t'a écoutée, Nina.
-papa|Tes mains sont au chaud.</t>
+          <t>narrateur|Les moufles reposent sur le radiateur.
+narrateur|Le petit nuage n'est plus là.
+enfant-f|L'éclat est là, papa.
+papa|Tu le vois sur le pouce ?
+enfant-f|Oui, papa.
+maman|On est bien, ici.
+narrateur|La soupe fume un peu, près de la fenêtre.
+narrateur|La fenêtre tremble moins.
+enfant-f|J'ai dit le secret.
+maman|On t'a entendue, Nina.
+enfant-f|Oui, maman.
+narrateur|Nina pose la joue près de la laine.
+narrateur|La laine est tiède, un peu rêche.
+enfant-f|C'est chaud.
+narrateur|Dehors, le froid reste sur les cailloux.
+narrateur|L'éclat de moufle tient sur le pouce.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>radiateur,laine</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2201,6 +2298,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>